<commit_message>
adicion de mas campos para los formularios
</commit_message>
<xml_diff>
--- a/src/main/resources/reports/plantilla_acta_v2.xlsx
+++ b/src/main/resources/reports/plantilla_acta_v2.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frank\Pictures\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C6A55D-D167-47E4-B190-36239E29A495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12720"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,12 +25,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Jorge F. Coaquira Ramos</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -44,7 +45,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0">
+    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -64,29 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6"/>
-        <color rgb="FF202429"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ENTIDAD U ORGANIZACIÓN DE LA ENTIDAD:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="6"/>
-        <color rgb="FF202429"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>CORTE SUPERIOR DE JUSTICIA DE AREQUIPA</t>
-    </r>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t>${fecha}</t>
   </si>
@@ -335,12 +314,49 @@
   <si>
     <t>${tipo}</t>
   </si>
+  <si>
+    <t>Control Patrimonial</t>
+  </si>
+  <si>
+    <t>${personalControlPatrimonial}</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="6"/>
+        <color rgb="FF202429"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>ENTIDAD U ORGANIZACIÓN DE LA ENTIDAD:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="6"/>
+        <color rgb="FF202429"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF202429"/>
+        <rFont val="Arial MT"/>
+      </rPr>
+      <t>CORTE SUPERIOR DE JUSTICIA DE AREQUIPA</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -407,12 +423,6 @@
     <font>
       <sz val="5"/>
       <color rgb="FF202429"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="5"/>
-      <color rgb="FF202429"/>
       <name val="Arial MT"/>
       <family val="2"/>
     </font>
@@ -463,6 +473,35 @@
       <color rgb="FF202429"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF202429"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Arial MT"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF202429"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF202429"/>
+      <name val="Arial MT"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color rgb="FF202429"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -639,7 +678,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -683,7 +722,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -695,113 +734,122 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="17"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="47"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="47"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1132,279 +1180,293 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.140625" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="37.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="9" max="9" width="39.5703125" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="3" width="40.21875" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="39.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
-      <c r="A1" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
+    <row r="1" spans="1:9" ht="15.6">
+      <c r="A1" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
     </row>
     <row r="2" spans="1:9" ht="44.25" customHeight="1">
-      <c r="A2" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="A2" s="57" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
       <c r="H2" s="1"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
-      <c r="A3" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
+      <c r="A3" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
       <c r="H3" s="17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I3" s="18" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="31" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="33"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="18" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="21" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="5"/>
+      <c r="I5" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="26" t="s">
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="31" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="21" t="s">
+      <c r="B6" s="32"/>
+      <c r="C6" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="23" t="s">
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="53"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="27"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="21" t="s">
+      <c r="B7" s="32"/>
+      <c r="C7" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="23" t="s">
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="39" t="s">
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="31" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="21" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="37"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="40"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="41" t="s">
+      <c r="B9" s="39"/>
+      <c r="C9" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="45" t="s">
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="40"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="12" spans="1:9" ht="15" customHeight="1">
+      <c r="A12" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="47"/>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="43"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="3"/>
-    </row>
-    <row r="12" spans="1:9" ht="15" customHeight="1">
-      <c r="A12" s="51" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="52"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
     </row>
     <row r="13" spans="1:9" ht="16.5" customHeight="1">
       <c r="A13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="C13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="G13" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="I13" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="12" t="s">
+    </row>
+    <row r="14" spans="1:9" ht="14.25" customHeight="1">
+      <c r="A14" s="19" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="14.25" customHeight="1">
-      <c r="A14" s="53" t="s">
+      <c r="B14" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="54" t="s">
+      <c r="C14" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="D14" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="53" t="s">
+      <c r="E14" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="53" t="s">
+      <c r="F14" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="53" t="s">
+      <c r="G14" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="53" t="s">
+      <c r="H14" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="H14" s="53" t="s">
+      <c r="I14" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="I14" s="53" t="s">
+    </row>
+    <row r="16" spans="1:9" ht="57.75" customHeight="1">
+      <c r="A16" s="54" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="57.75" customHeight="1">
-      <c r="A16" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="36"/>
-      <c r="I16" s="36"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
     </row>
     <row r="18" spans="3:8" ht="49.5" customHeight="1">
       <c r="C18" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
-      <c r="F18" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
+      <c r="F18" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
     </row>
     <row r="19" spans="3:8" ht="15" customHeight="1">
-      <c r="C19" s="16"/>
+      <c r="C19" s="56" t="s">
+        <v>43</v>
+      </c>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
-      <c r="F19" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="G19" s="29"/>
-      <c r="H19" s="30"/>
+      <c r="F19" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G19" s="22"/>
+      <c r="H19" s="23"/>
+    </row>
+    <row r="20" spans="3:8">
+      <c r="C20" s="55" t="s">
+        <v>42</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:H6"/>
     <mergeCell ref="F19:H19"/>
     <mergeCell ref="A3:G4"/>
     <mergeCell ref="A16:I16"/>
@@ -1417,13 +1479,6 @@
     <mergeCell ref="A9:B10"/>
     <mergeCell ref="C9:H10"/>
     <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="53" orientation="portrait" r:id="rId1"/>

</xml_diff>